<commit_message>
Added new measurements Excel file and found a new dead zone width
</commit_message>
<xml_diff>
--- a/Measurements/SpeedToPwm.xlsx
+++ b/Measurements/SpeedToPwm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13dae0734b4968e2/PoliTo/Tirocinio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Freenove4WD_TargetFollowing\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="394" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC279732-45A7-4C7E-A49D-2A8B87DFC6D2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C727024-CB3E-4CA6-AAA7-08AB9E651762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4800" yWindow="2152" windowWidth="14400" windowHeight="8183" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
   <si>
     <t>SPACE (cm)</t>
   </si>
@@ -55,6 +55,12 @@
   <si>
     <t>TIME_4W (s)</t>
   </si>
+  <si>
+    <t>2 FRONTAL WHEELS</t>
+  </si>
+  <si>
+    <t>4 WHEELS</t>
+  </si>
 </sst>
 </file>
 
@@ -63,7 +69,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,7 +86,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -151,11 +157,143 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -187,15 +325,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -360,10 +522,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$N$2:$N$7</c:f>
+              <c:f>Sheet1!$N$2:$N$12</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>21.34</c:v>
                 </c:pt>
@@ -381,16 +543,31 @@
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-21.34</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-26.64</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-50.26</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-55.96</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-66.14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$M$2:$M$7</c:f>
+              <c:f>Sheet1!$M$2:$M$12</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>720</c:v>
                 </c:pt>
@@ -408,6 +585,21 @@
                 </c:pt>
                 <c:pt idx="5" formatCode="General">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-720</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-1023</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2047</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3071</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4095</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -788,7 +980,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14689760130372825"/>
+          <c:y val="0.13171418896492446"/>
+          <c:w val="0.81630648487127733"/>
+          <c:h val="0.77522634736767637"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -908,10 +1110,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$M$2:$M$7</c:f>
+              <c:f>Sheet1!$M$2:$M$12</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>720</c:v>
                 </c:pt>
@@ -929,16 +1131,31 @@
                 </c:pt>
                 <c:pt idx="5" formatCode="General">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-720</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-1023</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2047</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3071</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4095</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$N$2:$N$7</c:f>
+              <c:f>Sheet1!$N$2:$N$12</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>21.34</c:v>
                 </c:pt>
@@ -956,6 +1173,21 @@
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-21.34</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-26.64</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-50.26</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-55.96</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-66.14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -964,6 +1196,1128 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-E3C1-4CC9-9631-7912AA08A815}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="750332423"/>
+        <c:axId val="750334471"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="750332423"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>PWM</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750334471"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="750334471"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>cm/s</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="5.9474665429417361E-3"/>
+              <c:y val="0.45532143299572025"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750332423"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>SpeedToPWM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="3"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$O$2:$O$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>21.79</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>35.89</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>61.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>72.87</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>80.78</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-21.79</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-35.89</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-61.82</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-72.87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-80.78</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$M$2:$M$12</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>720</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1023</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2047</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3071</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4095</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-720</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-1023</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2047</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3071</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4095</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-EE6B-4F0E-8C7E-6C9E11E5878D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="750332423"/>
+        <c:axId val="750334471"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="750332423"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>cm/s</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750334471"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="750334471"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>PWM</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="5.9474665429417361E-3"/>
+              <c:y val="0.45532143299572025"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="750332423"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>PWMtoSpeed</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.14689760130372825"/>
+          <c:y val="0.13171418896492446"/>
+          <c:w val="0.81630648487127733"/>
+          <c:h val="0.77522634736767637"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="3"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$M$2:$M$12</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>720</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1023</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2047</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3071</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4095</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-720</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-1023</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-2047</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3071</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-4095</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$O$2:$O$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>21.79</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>35.89</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>61.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>72.87</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>80.78</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-21.79</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-35.89</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-61.82</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-72.87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-80.78</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A151-43AC-8C5B-9E32C37AE568}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1345,6 +2699,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1862,6 +3296,1038 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2382,15 +4848,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
+      <xdr:colOff>83344</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>590550</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>560784</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>69057</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2417,16 +4883,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>233869</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>520809</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>78582</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2451,6 +4917,85 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83344</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>560784</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>69057</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC465855-879C-459E-B839-4844FB20DDDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>233869</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>520809</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>78582</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEB03672-D77C-4BC9-9E12-49C7F9551DC0}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{9918C293-6F6E-2184-C495-C6849CADF1C2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2776,17 +5321,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:Q59"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="13" max="13" width="12.85546875" customWidth="1"/>
-    <col min="14" max="15" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.59765625" customWidth="1"/>
+    <col min="2" max="2" width="13.3984375" customWidth="1"/>
+    <col min="3" max="3" width="10.1328125" customWidth="1"/>
+    <col min="13" max="13" width="12.86328125" customWidth="1"/>
+    <col min="14" max="15" width="17.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="20.25" customHeight="1">
+    <row r="1" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -2813,7 +5358,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2833,9 +5378,12 @@
         <f>ROUND(B1/AVERAGE(C12:K12), 2)</f>
         <v>21.34</v>
       </c>
-      <c r="O2" s="8"/>
+      <c r="O2" s="8">
+        <f>ROUND(B1/AVERAGE(C13:K13), 2)</f>
+        <v>21.79</v>
+      </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
@@ -2857,10 +5405,13 @@
         <f>ROUND(B1/AVERAGE(C10:K10), 2)</f>
         <v>26.64</v>
       </c>
-      <c r="O3" s="8"/>
+      <c r="O3" s="8">
+        <f>ROUND(B1/AVERAGE(C11:K11), 2)</f>
+        <v>35.89</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="16.5" customHeight="1">
-      <c r="A4" s="11">
+    <row r="4" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="14">
         <v>4095</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -2901,22 +5452,43 @@
         <f>ROUND(B1/AVERAGE(C8:K8), 2)</f>
         <v>50.26</v>
       </c>
-      <c r="O4" s="8"/>
+      <c r="O4" s="8">
+        <f>ROUND(B1/AVERAGE(C9:K9), 2)</f>
+        <v>61.82</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" ht="17.25" customHeight="1">
-      <c r="A5" s="12"/>
+    <row r="5" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="15"/>
       <c r="B5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="C5" s="8">
+        <v>1.45</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.51</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1.48</v>
+      </c>
+      <c r="F5" s="8">
+        <v>1.59</v>
+      </c>
+      <c r="G5" s="8">
+        <v>1.41</v>
+      </c>
+      <c r="H5" s="8">
+        <v>1.54</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1.45</v>
+      </c>
+      <c r="J5" s="8">
+        <v>1.45</v>
+      </c>
+      <c r="K5" s="8">
+        <v>1.49</v>
+      </c>
       <c r="L5" s="3"/>
       <c r="M5" s="9">
         <v>3071</v>
@@ -2925,10 +5497,13 @@
         <f>ROUND(B1/AVERAGE(C6:K6), 2)</f>
         <v>55.96</v>
       </c>
-      <c r="O5" s="8"/>
+      <c r="O5" s="8">
+        <f>ROUND(B1/AVERAGE(C7:K7), 2)</f>
+        <v>72.87</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A6" s="11">
+    <row r="6" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="14">
         <v>3071</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -2962,29 +5537,50 @@
         <v>2.14</v>
       </c>
       <c r="L6" s="3"/>
-      <c r="M6" s="13">
+      <c r="M6" s="11">
         <v>4095</v>
       </c>
       <c r="N6" s="7">
         <f>ROUND(B1/AVERAGE(C4:K4), 2)</f>
         <v>66.14</v>
       </c>
-      <c r="O6" s="7"/>
+      <c r="O6" s="7">
+        <f>ROUND(B1/AVERAGE(C5:K5), 2)</f>
+        <v>80.78</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" ht="19.5" customHeight="1">
-      <c r="A7" s="11"/>
+    <row r="7" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="14"/>
       <c r="B7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="C7" s="8">
+        <v>1.62</v>
+      </c>
+      <c r="D7" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1.71</v>
+      </c>
+      <c r="F7" s="8">
+        <v>1.56</v>
+      </c>
+      <c r="G7" s="8">
+        <v>1.64</v>
+      </c>
+      <c r="H7" s="8">
+        <v>1.66</v>
+      </c>
+      <c r="I7" s="8">
+        <v>1.68</v>
+      </c>
+      <c r="J7" s="8">
+        <v>1.66</v>
+      </c>
+      <c r="K7" s="8">
+        <v>1.59</v>
+      </c>
       <c r="L7" s="3"/>
       <c r="M7" s="10">
         <v>0</v>
@@ -2992,10 +5588,12 @@
       <c r="N7" s="8">
         <v>0</v>
       </c>
-      <c r="O7" s="10"/>
+      <c r="O7" s="8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A8" s="11">
+    <row r="8" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="14">
         <f>M4</f>
         <v>2047</v>
       </c>
@@ -3029,24 +5627,64 @@
       <c r="K8" s="8">
         <v>2.4700000000000002</v>
       </c>
+      <c r="M8" s="9">
+        <v>-720</v>
+      </c>
+      <c r="N8" s="8">
+        <f>-N2</f>
+        <v>-21.34</v>
+      </c>
+      <c r="O8" s="8">
+        <f>-O2</f>
+        <v>-21.79</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A9" s="11"/>
+    <row r="9" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="14"/>
       <c r="B9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
+      <c r="C9" s="8">
+        <v>1.98</v>
+      </c>
+      <c r="D9" s="8">
+        <v>1.94</v>
+      </c>
+      <c r="E9" s="8">
+        <v>1.94</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1.93</v>
+      </c>
+      <c r="G9" s="8">
+        <v>1.95</v>
+      </c>
+      <c r="H9" s="8">
+        <v>1.91</v>
+      </c>
+      <c r="I9" s="8">
+        <v>1.93</v>
+      </c>
+      <c r="J9" s="8">
+        <v>1.97</v>
+      </c>
+      <c r="K9" s="8">
+        <v>1.92</v>
+      </c>
+      <c r="M9" s="9">
+        <v>-1023</v>
+      </c>
+      <c r="N9" s="8">
+        <f>-N3</f>
+        <v>-26.64</v>
+      </c>
+      <c r="O9" s="8">
+        <f>-O3</f>
+        <v>-35.89</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A10" s="11">
+    <row r="10" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="14">
         <v>1023</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -3079,24 +5717,64 @@
       <c r="K10" s="8">
         <v>4.4400000000000004</v>
       </c>
+      <c r="M10" s="9">
+        <v>-2047</v>
+      </c>
+      <c r="N10" s="8">
+        <f>-N4</f>
+        <v>-50.26</v>
+      </c>
+      <c r="O10" s="8">
+        <f>-O4</f>
+        <v>-61.82</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" ht="20.25" customHeight="1">
-      <c r="A11" s="11"/>
+    <row r="11" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="14"/>
       <c r="B11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
+      <c r="C11" s="8">
+        <v>3.32</v>
+      </c>
+      <c r="D11" s="8">
+        <v>3.38</v>
+      </c>
+      <c r="E11" s="8">
+        <v>3.32</v>
+      </c>
+      <c r="F11" s="8">
+        <v>3.31</v>
+      </c>
+      <c r="G11" s="8">
+        <v>3.34</v>
+      </c>
+      <c r="H11" s="8">
+        <v>3.42</v>
+      </c>
+      <c r="I11" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="J11" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="K11" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="M11" s="9">
+        <v>-3071</v>
+      </c>
+      <c r="N11" s="8">
+        <f>-N5</f>
+        <v>-55.96</v>
+      </c>
+      <c r="O11" s="8">
+        <f>-O5</f>
+        <v>-72.87</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" ht="15">
-      <c r="A12" s="11">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A12" s="14">
         <v>720</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -3129,25 +5807,897 @@
       <c r="K12" s="8">
         <v>5.9</v>
       </c>
+      <c r="M12" s="12">
+        <v>-4095</v>
+      </c>
+      <c r="N12" s="13">
+        <f>-N6</f>
+        <v>-66.14</v>
+      </c>
+      <c r="O12" s="13">
+        <f>-O6</f>
+        <v>-80.78</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A13" s="11"/>
+    <row r="13" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="14"/>
       <c r="B13" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
+      <c r="C13" s="8">
+        <v>5.79</v>
+      </c>
+      <c r="D13" s="8">
+        <v>5.55</v>
+      </c>
+      <c r="E13" s="8">
+        <v>5.42</v>
+      </c>
+      <c r="F13" s="8">
+        <v>5.49</v>
+      </c>
+      <c r="G13" s="8">
+        <v>5.52</v>
+      </c>
+      <c r="H13" s="8">
+        <v>5.43</v>
+      </c>
+      <c r="I13" s="8">
+        <v>5.46</v>
+      </c>
+      <c r="J13" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="K13" s="8">
+        <v>5.41</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" ht="19.5" customHeight="1"/>
+    <row r="14" spans="1:17" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="15" spans="1:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="18"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A16" s="19"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="20"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="21"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A17" s="22"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="24"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A18" s="22"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="24"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="23"/>
+      <c r="Q19" s="24"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A20" s="22"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="23"/>
+      <c r="O20" s="23"/>
+      <c r="P20" s="23"/>
+      <c r="Q20" s="24"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A21" s="22"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="23"/>
+      <c r="Q21" s="24"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A22" s="22"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
+      <c r="O22" s="23"/>
+      <c r="P22" s="23"/>
+      <c r="Q22" s="24"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A23" s="22"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="23"/>
+      <c r="O23" s="23"/>
+      <c r="P23" s="23"/>
+      <c r="Q23" s="24"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A24" s="22"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="23"/>
+      <c r="O24" s="23"/>
+      <c r="P24" s="23"/>
+      <c r="Q24" s="24"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A25" s="22"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="23"/>
+      <c r="Q25" s="24"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A26" s="22"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="24"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A27" s="22"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="24"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A28" s="22"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="24"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A29" s="22"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
+      <c r="P29" s="23"/>
+      <c r="Q29" s="24"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A30" s="22"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
+      <c r="P30" s="23"/>
+      <c r="Q30" s="24"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A31" s="22"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+      <c r="P31" s="23"/>
+      <c r="Q31" s="24"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A32" s="22"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
+      <c r="P32" s="23"/>
+      <c r="Q32" s="24"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A33" s="22"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="23"/>
+      <c r="N33" s="23"/>
+      <c r="O33" s="23"/>
+      <c r="P33" s="23"/>
+      <c r="Q33" s="24"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A34" s="22"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+      <c r="N34" s="23"/>
+      <c r="O34" s="23"/>
+      <c r="P34" s="23"/>
+      <c r="Q34" s="24"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A35" s="22"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
+      <c r="P35" s="23"/>
+      <c r="Q35" s="24"/>
+    </row>
+    <row r="36" spans="1:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A36" s="25"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="26"/>
+      <c r="L36" s="26"/>
+      <c r="M36" s="26"/>
+      <c r="N36" s="26"/>
+      <c r="O36" s="26"/>
+      <c r="P36" s="26"/>
+      <c r="Q36" s="27"/>
+    </row>
+    <row r="37" spans="1:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="38" spans="1:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A38" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="N38" s="17"/>
+      <c r="O38" s="17"/>
+      <c r="P38" s="17"/>
+      <c r="Q38" s="18"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A39" s="19"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="20"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
+      <c r="O39" s="20"/>
+      <c r="P39" s="20"/>
+      <c r="Q39" s="21"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A40" s="22"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23"/>
+      <c r="Q40" s="24"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A41" s="22"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="24"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A42" s="22"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="23"/>
+      <c r="Q42" s="24"/>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A43" s="22"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="23"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="23"/>
+      <c r="K43" s="23"/>
+      <c r="L43" s="23"/>
+      <c r="M43" s="23"/>
+      <c r="N43" s="23"/>
+      <c r="O43" s="23"/>
+      <c r="P43" s="23"/>
+      <c r="Q43" s="24"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A44" s="22"/>
+      <c r="B44" s="23"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="23"/>
+      <c r="E44" s="23"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23"/>
+      <c r="K44" s="23"/>
+      <c r="L44" s="23"/>
+      <c r="M44" s="23"/>
+      <c r="N44" s="23"/>
+      <c r="O44" s="23"/>
+      <c r="P44" s="23"/>
+      <c r="Q44" s="24"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A45" s="22"/>
+      <c r="B45" s="23"/>
+      <c r="C45" s="23"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23"/>
+      <c r="K45" s="23"/>
+      <c r="L45" s="23"/>
+      <c r="M45" s="23"/>
+      <c r="N45" s="23"/>
+      <c r="O45" s="23"/>
+      <c r="P45" s="23"/>
+      <c r="Q45" s="24"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A46" s="22"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
+      <c r="M46" s="23"/>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+      <c r="P46" s="23"/>
+      <c r="Q46" s="24"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A47" s="22"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23"/>
+      <c r="M47" s="23"/>
+      <c r="N47" s="23"/>
+      <c r="O47" s="23"/>
+      <c r="P47" s="23"/>
+      <c r="Q47" s="24"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A48" s="22"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="23"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
+      <c r="M48" s="23"/>
+      <c r="N48" s="23"/>
+      <c r="O48" s="23"/>
+      <c r="P48" s="23"/>
+      <c r="Q48" s="24"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A49" s="22"/>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="23"/>
+      <c r="H49" s="23"/>
+      <c r="I49" s="23"/>
+      <c r="J49" s="23"/>
+      <c r="K49" s="23"/>
+      <c r="L49" s="23"/>
+      <c r="M49" s="23"/>
+      <c r="N49" s="23"/>
+      <c r="O49" s="23"/>
+      <c r="P49" s="23"/>
+      <c r="Q49" s="24"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A50" s="22"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="23"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
+      <c r="M50" s="23"/>
+      <c r="N50" s="23"/>
+      <c r="O50" s="23"/>
+      <c r="P50" s="23"/>
+      <c r="Q50" s="24"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A51" s="22"/>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="23"/>
+      <c r="J51" s="23"/>
+      <c r="K51" s="23"/>
+      <c r="L51" s="23"/>
+      <c r="M51" s="23"/>
+      <c r="N51" s="23"/>
+      <c r="O51" s="23"/>
+      <c r="P51" s="23"/>
+      <c r="Q51" s="24"/>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A52" s="22"/>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="23"/>
+      <c r="O52" s="23"/>
+      <c r="P52" s="23"/>
+      <c r="Q52" s="24"/>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A53" s="22"/>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="23"/>
+      <c r="J53" s="23"/>
+      <c r="K53" s="23"/>
+      <c r="L53" s="23"/>
+      <c r="M53" s="23"/>
+      <c r="N53" s="23"/>
+      <c r="O53" s="23"/>
+      <c r="P53" s="23"/>
+      <c r="Q53" s="24"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A54" s="22"/>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="23"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="23"/>
+      <c r="K54" s="23"/>
+      <c r="L54" s="23"/>
+      <c r="M54" s="23"/>
+      <c r="N54" s="23"/>
+      <c r="O54" s="23"/>
+      <c r="P54" s="23"/>
+      <c r="Q54" s="24"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A55" s="22"/>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
+      <c r="J55" s="23"/>
+      <c r="K55" s="23"/>
+      <c r="L55" s="23"/>
+      <c r="M55" s="23"/>
+      <c r="N55" s="23"/>
+      <c r="O55" s="23"/>
+      <c r="P55" s="23"/>
+      <c r="Q55" s="24"/>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A56" s="22"/>
+      <c r="B56" s="23"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
+      <c r="H56" s="23"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="23"/>
+      <c r="K56" s="23"/>
+      <c r="L56" s="23"/>
+      <c r="M56" s="23"/>
+      <c r="N56" s="23"/>
+      <c r="O56" s="23"/>
+      <c r="P56" s="23"/>
+      <c r="Q56" s="24"/>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A57" s="22"/>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="23"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="23"/>
+      <c r="H57" s="23"/>
+      <c r="I57" s="23"/>
+      <c r="J57" s="23"/>
+      <c r="K57" s="23"/>
+      <c r="L57" s="23"/>
+      <c r="M57" s="23"/>
+      <c r="N57" s="23"/>
+      <c r="O57" s="23"/>
+      <c r="P57" s="23"/>
+      <c r="Q57" s="24"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="A58" s="22"/>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="23"/>
+      <c r="H58" s="23"/>
+      <c r="I58" s="23"/>
+      <c r="J58" s="23"/>
+      <c r="K58" s="23"/>
+      <c r="L58" s="23"/>
+      <c r="M58" s="23"/>
+      <c r="N58" s="23"/>
+      <c r="O58" s="23"/>
+      <c r="P58" s="23"/>
+      <c r="Q58" s="24"/>
+    </row>
+    <row r="59" spans="1:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A59" s="25"/>
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="26"/>
+      <c r="I59" s="26"/>
+      <c r="J59" s="26"/>
+      <c r="K59" s="26"/>
+      <c r="L59" s="26"/>
+      <c r="M59" s="26"/>
+      <c r="N59" s="26"/>
+      <c r="O59" s="26"/>
+      <c r="P59" s="26"/>
+      <c r="Q59" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="A15:Q15"/>
+    <mergeCell ref="A38:Q38"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A8:A9"/>

</xml_diff>